<commit_message>
updated raw data AND new output csvs
</commit_message>
<xml_diff>
--- a/Results/MainExperiment/DataFormatting-and-Audio/dataOutput/audioTranscriptFiltered.xlsx
+++ b/Results/MainExperiment/DataFormatting-and-Audio/dataOutput/audioTranscriptFiltered.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="207">
   <si>
     <t xml:space="preserve">participant</t>
   </si>
@@ -497,6 +497,150 @@
   </si>
   <si>
     <t xml:space="preserve">for this one in particular i chose to do the slider at 100 i'm just because it was the only one that had any type of similarity to angry whereas the other ones were happy or just a blank face</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6980dfb784202dcf9736910f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i chose to put them in that position because like i think five stars would be excellent and two stars would probably be closer to bad so 4 stars i thought with what was left would either be technical dramatic or good so as a result i think 4 stars being good makes the most sense but because i guess you could you know have a highly critical person say 5 stars is just good or you know not critical person at all say two stars it's bad or two stars is good that's why i had a little room for margin error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">69d5c4d748bcaf8026c80573</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the word i choose is stupid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i chose four star because five star would have been excellent and so 4 star is good</t>
+  </si>
+  <si>
+    <t xml:space="preserve">69864a705614c15728117b35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">where do i choose is first</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I think I put the sliders that I did because I mean there’s only happy neutral and mad, so I mean, yea that’s pretty like you can just see that essentially</t>
+  </si>
+  <si>
+    <t xml:space="preserve">65465c5bc5a014ec683d55cf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i chose this because the person speaking said good and looking at the three options there are two stars four stars then five stars and looking at the options of words excellent would be the best word i would think so i would say that that would be five stars and bad would be two stars so good seem like a good midway answer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6a00b4c7593a89490830c18c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the reason why i chose fat and put 100 on it is because the question asked which image and there was the there was quiet thin monstrous obese or fat and he's a fat and he didn’t say obese or monstrous</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6a15dfdb880253e5b6b917f3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the word i choose is 9th</t>
+  </si>
+  <si>
+    <t xml:space="preserve">because you said good not great</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6a04948f1e40214a25ff2563</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i put my sliders in that position because both two and three could be considered fat but three can also be considered obese but it but because the word i was given by the recording was fat it could be two or three because both would be considered fat but three would also be considered obese</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6a1582166cefcdcbed565058</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the word i choose here is first</t>
+  </si>
+  <si>
+    <t xml:space="preserve">what a word i choose here is tied</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i chose to put the slider in this one because this is the only face that looked angry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">69b19e44edf4d70aee145c16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i chose to put the sliders in those positions based on what the what the participants said and that it matched the words based on what the participant said</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6a14c736578656591db6ea31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i'm not really sure what this person considers to be fat as that's kind of an objective thing versus a word like obese which has a more concrete definition so that's why i came to the sliders like that because i'm not sure how they define that word</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6a15d5fb80117206e7200cf7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chose the last one because the first two photos do not look angry the first photo looks neutral the second photo looks happy or just in a better mood and then the third one looks displeased so i figured the third one would be most correct for the angry face or angry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">69e599577d00fb31c54fb004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the word I choose is first</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I think it was fairly clear what they were trying to convey from the words they chose and if we’re looking at this one specifically, it could’ve been three or four, just because five stars is great and 4 stars is good. it could’ve been either or</t>
+  </si>
+  <si>
+    <t xml:space="preserve">699d45af20adaa6e1e89aa5a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">she is the only one that looks angry to me so that is why i decided to give that one the full 100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6a0dbb470d44c02c7ec444f0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">some of them had a responses that could go between the two of the selections however i tried to choose the one that was probably most apt but they was still a little bit of doubt left that i usually had a little bit more for the other option</t>
+  </si>
+  <si>
+    <t xml:space="preserve">697a495862ac67423e8418b8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">69b3193cce0978ad6db9fe7c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">decided to put the slider at 100% for the four stars because excellent would have been five stars and bad would have been two stars and it's not those two</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6a0b7296246f70341f078e55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">looking at the words i see thin which probably correlates to one fat which correlates to two and obese which would correlate to 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6a0e0a9490e868c044e21936</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I put the slider in the box with the four stars because frank said i think his name is frank frank or eric said that the word he chose was good and since there are options of bad good in excellent i used the middle option</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6a0f1056788a67850f057de4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">because good is 4 stars excellent is 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">69fd3605435216c2d93bc72f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i chose the positions but i did because i feel like if they were describe the biggest person they would have chose monstrous or maybe obese and if it were the first person they would have chose quaint or thin however because monstrous and obese are extreme sides of the scale and they didn't say either of those i assume that it was the middle one and not the thing or quaint one</t>
+  </si>
+  <si>
+    <t xml:space="preserve">665795d82a087799023aaf0e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the word I choose is tied</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i felt that the pictures and the words that they spoke, the picture i chose represented the word that they spoke</t>
   </si>
 </sst>
 </file>
@@ -511,6 +655,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -582,7 +727,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -600,6 +745,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -680,14 +837,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E66"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E87"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="23.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="27.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="21.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="38.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="27.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1140,7 +1297,7 @@
       <c r="D27" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" s="3" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1803,6 +1960,361 @@
       </c>
       <c r="E66" s="3" t="s">
         <v>158</v>
+      </c>
+    </row>
+    <row r="67" s="5" customFormat="true" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="5" t="n">
+        <v>78</v>
+      </c>
+      <c r="B67" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="C67" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D67" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="68" s="5" customFormat="true" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="5" t="n">
+        <v>79</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C68" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D68" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="B69" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="C69" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="D69" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="E69" s="7" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="6" t="n">
+        <v>81</v>
+      </c>
+      <c r="B70" s="0" t="s">
+        <v>167</v>
+      </c>
+      <c r="C70" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D70" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="E70" s="7" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="B71" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="C71" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D71" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="E71" s="7" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="72" s="5" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="5" t="n">
+        <v>83</v>
+      </c>
+      <c r="B72" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="C72" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="D72" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="B73" s="0" t="s">
+        <v>174</v>
+      </c>
+      <c r="C73" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D73" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="E73" s="7" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="B74" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="C74" s="0" t="s">
+        <v>177</v>
+      </c>
+      <c r="D74" s="0" t="s">
+        <v>178</v>
+      </c>
+      <c r="E74" s="7" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="6" t="n">
+        <v>86</v>
+      </c>
+      <c r="B75" s="0" t="s">
+        <v>180</v>
+      </c>
+      <c r="C75" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D75" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="E75" s="7" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="6" t="n">
+        <v>87</v>
+      </c>
+      <c r="B76" s="0" t="s">
+        <v>182</v>
+      </c>
+      <c r="C76" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="D76" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="E76" s="7" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="6" t="n">
+        <v>88</v>
+      </c>
+      <c r="B77" s="0" t="s">
+        <v>184</v>
+      </c>
+      <c r="C77" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D77" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="E77" s="7" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="6" t="n">
+        <v>89</v>
+      </c>
+      <c r="B78" s="0" t="s">
+        <v>186</v>
+      </c>
+      <c r="C78" s="0" t="s">
+        <v>187</v>
+      </c>
+      <c r="D78" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="E78" s="7" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="B79" s="0" t="s">
+        <v>189</v>
+      </c>
+      <c r="C79" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D79" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="E79" s="7" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="6" t="n">
+        <v>91</v>
+      </c>
+      <c r="B80" s="0" t="s">
+        <v>191</v>
+      </c>
+      <c r="C80" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D80" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="E80" s="7" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="81" s="5" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="5" t="n">
+        <v>92</v>
+      </c>
+      <c r="B81" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="C81" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D81" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E81" s="3"/>
+    </row>
+    <row r="82" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="6" t="n">
+        <v>93</v>
+      </c>
+      <c r="B82" s="0" t="s">
+        <v>194</v>
+      </c>
+      <c r="C82" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="D82" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="E82" s="7" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="6" t="n">
+        <v>94</v>
+      </c>
+      <c r="B83" s="0" t="s">
+        <v>196</v>
+      </c>
+      <c r="C83" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="D83" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="E83" s="7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="6" t="n">
+        <v>95</v>
+      </c>
+      <c r="B84" s="0" t="s">
+        <v>198</v>
+      </c>
+      <c r="C84" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D84" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="E84" s="7" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="6" t="n">
+        <v>96</v>
+      </c>
+      <c r="B85" s="0" t="s">
+        <v>200</v>
+      </c>
+      <c r="C85" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D85" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="E85" s="7" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="6" t="n">
+        <v>97</v>
+      </c>
+      <c r="B86" s="0" t="s">
+        <v>202</v>
+      </c>
+      <c r="C86" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D86" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="E86" s="7" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="6" t="n">
+        <v>98</v>
+      </c>
+      <c r="B87" s="0" t="s">
+        <v>204</v>
+      </c>
+      <c r="C87" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D87" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="E87" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>